<commit_message>
feat: Add support for BBVA Mastercard XLSX format
</commit_message>
<xml_diff>
--- a/temp/BBVA_MASTERCARD_20250315.xlsx
+++ b/temp/BBVA_MASTERCARD_20250315.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,21 +458,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-03-15</t>
+          <t>2025-07-07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ON FIT C.02/06 006805</t>
+          <t>Onlyfans.Com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ARS</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>107970</v>
+        <v>35</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -483,12 +483,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-03-27</t>
+          <t>2025-03-15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MERPAGO*MCDONALDS 927266</t>
+          <t>ON FIT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -497,109 +497,9 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4000</v>
+        <v>107970</v>
       </c>
       <c r="E3" t="inlineStr">
-        <is>
-          <t>BBVA Mastercard</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-03-27</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>MI GUSTO 007595</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>21000</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>BBVA Mastercard</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-03-28</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MERPAGO*SCANNAPIECO 978346</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>9500</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>BBVA Mastercard</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-03-29</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ASUMARE PALERMO-ASU MA 000046</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>39500</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>BBVA Mastercard</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-03-29</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>MERPAGO*MCDONALDSECOMM 879024</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>3200</v>
-      </c>
-      <c r="E7" t="inlineStr">
         <is>
           <t>BBVA Mastercard</t>
         </is>

</xml_diff>